<commit_message>
Update IG to version 0.1.2
Add a bundle with two reports, both without AI.
Correct some, not all, spelling mistakes.
Rename example instances consistently.
Replace all example GUIDs with proper GUIDs.
Add a example patients in separate files.
Fix CodeSystems SHOULD have a stated value for the caseSensitive and experimental
Fix Published value sets SHOULD conform to the ShareableValueSet profile, which says that the element ValueSet.experimental is mandatory.
Fix Structures referring to experimental things should also be experimental.
Fix Context warning for all extensions
Add documentation to the image-quality code system.
Add system for not-asked code system.
Add system for retina-examination-id and retina-observation-id.
Ignore warnings about not able to validate no-kodeverk-7275 or urn:oid:2.16.578.1.12.4.1.4.1
Ignore warning about elementdefinition-maxValueSet being deprecated.
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-conclusioncode-cs.xlsx
+++ b/docs/CodeSystem-retina-conclusioncode-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.1</t>
+    <t>0.1.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -54,10 +54,13 @@
     <t>Experimental</t>
   </si>
   <si>
+    <t>true</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-07T21:19:45+02:00</t>
+    <t>2025-10-19T20:08:40+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -343,110 +346,114 @@
       <c r="A7" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" t="s" s="2">
+        <v>13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>25</v>
-      </c>
-      <c r="B15" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -461,51 +468,51 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D4" s="2"/>
     </row>

</xml_diff>